<commit_message>
Updated Old File Submissions
</commit_message>
<xml_diff>
--- a/CIS 4374 Gantt Chart.xlsx
+++ b/CIS 4374 Gantt Chart.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\College Crap\Fall 2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Stuff from D Drive\College Crap\Fall 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB0C2860-4BBE-4330-9D47-09E2F791CF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC83402E-EB77-465A-92BA-872FD84929E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{61A1D63B-DCB9-44D3-B3A6-545F6DED8932}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt Chart" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">'Gantt Chart'!$A$1:$I$16</definedName>
@@ -48,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="34">
   <si>
     <t>Outline Level</t>
   </si>
@@ -141,6 +140,15 @@
   </si>
   <si>
     <t>Stocks And Bonds Management Software</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>Purple</t>
   </si>
 </sst>
 </file>
@@ -176,9 +184,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1880,19 +1887,24 @@
       <c r="B2">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>30</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>45918</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45993</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2">
         <v>76</v>
       </c>
-      <c r="H2" s="1"/>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -1901,26 +1913,26 @@
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>45918</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45931</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3">
         <v>14</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" t="s">
         <v>10</v>
       </c>
-      <c r="I3">
-        <v>31</v>
+      <c r="I3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1930,26 +1942,26 @@
       <c r="B4">
         <v>2</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45918</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45924</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4">
         <v>7</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" t="s">
         <v>10</v>
       </c>
-      <c r="I4">
-        <v>31</v>
+      <c r="I4" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -1959,26 +1971,26 @@
       <c r="B5">
         <v>3</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>45925</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45931</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5">
         <v>7</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" t="s">
         <v>13</v>
       </c>
-      <c r="I5">
-        <v>31</v>
+      <c r="I5" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1989,26 +2001,26 @@
         <f>B5+1</f>
         <v>4</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>45932</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45957</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6">
         <v>26</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" t="s">
         <v>10</v>
       </c>
-      <c r="I6">
-        <v>91</v>
+      <c r="I6" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -2019,26 +2031,26 @@
         <f t="shared" ref="B7:B16" si="0">B6+1</f>
         <v>5</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>45932</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45940</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7">
         <v>9</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" t="s">
         <v>10</v>
       </c>
-      <c r="I7">
-        <v>91</v>
+      <c r="I7" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -2049,26 +2061,26 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>45941</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45949</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8">
         <v>9</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" t="s">
         <v>25</v>
       </c>
-      <c r="I8">
-        <v>91</v>
+      <c r="I8" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -2079,26 +2091,26 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <v>45950</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9">
         <v>8</v>
       </c>
       <c r="G9">
         <v>0</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" t="s">
         <v>26</v>
       </c>
-      <c r="I9">
-        <v>91</v>
+      <c r="I9" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -2109,26 +2121,26 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>45958</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45981</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10">
         <v>24</v>
       </c>
       <c r="G10">
         <v>0</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" t="s">
         <v>10</v>
       </c>
-      <c r="I10">
-        <v>181</v>
+      <c r="I10" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -2139,26 +2151,26 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>45958</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>45965</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11">
         <v>8</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" t="s">
         <v>10</v>
       </c>
-      <c r="I11">
-        <v>181</v>
+      <c r="I11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -2169,26 +2181,26 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45966</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>45973</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12">
         <v>8</v>
       </c>
       <c r="G12">
         <v>0</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="H12" t="s">
         <v>27</v>
       </c>
-      <c r="I12">
-        <v>181</v>
+      <c r="I12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -2199,26 +2211,26 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45974</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>45981</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13">
         <v>8</v>
       </c>
       <c r="G13">
         <v>0</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" t="s">
         <v>28</v>
       </c>
-      <c r="I13">
-        <v>181</v>
+      <c r="I13" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -2229,26 +2241,26 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45982</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>45993</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14">
         <v>12</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" t="s">
         <v>10</v>
       </c>
-      <c r="I14">
-        <v>211</v>
+      <c r="I14" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -2259,26 +2271,26 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>45982</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>45985</v>
       </c>
-      <c r="F15" s="1">
+      <c r="F15">
         <v>4</v>
       </c>
       <c r="G15">
         <v>0</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="H15" t="s">
         <v>10</v>
       </c>
-      <c r="I15">
-        <v>211</v>
+      <c r="I15" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -2289,26 +2301,26 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45986</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>45993</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16">
         <v>8</v>
       </c>
       <c r="G16">
         <v>0</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="H16" t="s">
         <v>29</v>
       </c>
-      <c r="I16">
-        <v>211</v>
+      <c r="I16" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2317,15 +2329,6 @@
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F27746-AE06-417C-AE24-50E1FF7D8C31}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>